<commit_message>
Update notebooks, Excel report, and charts after verification
</commit_message>
<xml_diff>
--- a/output/NHS_AE_Report.xlsx
+++ b/output/NHS_AE_Report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics Program Lumen Digital Munich\Module#4 Python\Lesson#12\nhs-ae-analytics\outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics Program Lumen Digital Munich\Module#4 Python\Lesson#12\nhs-ae-analytics\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1D24FF6-1CF1-49AE-8C4B-D7162F00D884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7134BA48-D0F6-4FE1-AD21-26D0B9162654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="778" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="779" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Title Page" sheetId="1" r:id="rId1"/>
@@ -88,7 +88,7 @@
     <t>1,041 rows flagged (1.10%) retained in dataset, excluded from aggregations via SUPPRESSION != "Y" filter at analysis time, not dropped</t>
   </si>
   <si>
-    <t>After removing ENGLAND aggregate (Lesson 4)</t>
+    <t>After removing ENGLAND aggregate</t>
   </si>
   <si>
     <t>575 rows removed (25 months x 23 KPIs)</t>
@@ -109,7 +109,7 @@
     <t>After filtering to active NHS Trusts only</t>
   </si>
   <si>
-    <t>140 active NHS Trusts with submissions; 65 active Trusts made no submissions in period; 56 non-Trust orgs and 68 closed Trusts excluded</t>
+    <t>140 active NHS Trusts with submissions; 56 non-Trust orgs and 68 closed Trusts excluded</t>
   </si>
   <si>
     <t>Check</t>
@@ -202,7 +202,7 @@
     <t>Analytical population df_final</t>
   </si>
   <si>
-    <t>78,386 rows; 140 active NHS Trusts with submissions; 65 active Trusts in register made no submissions in period</t>
+    <t>78,386 rows; 140 active NHS Trusts with submissions</t>
   </si>
   <si>
     <t>Three filters applied: ENG aggregate removed, closed Trusts removed, non-Trust providers removed</t>
@@ -1309,7 +1309,7 @@
     <t>National A&amp;E wait times peaked at 186 minutes in December 2023 and have stabilised in a tighter 159–167 minute range since spring 2025.</t>
   </si>
   <si>
-    <t>Faster treatment times show no meaningful link to lower reattendance rates, two Trusts with the fastest treatment times actually have the highest reattendance rates in the dataset.</t>
+    <t>Faster treatment times show no meaningful link to lower reattendance rates, two Trusts (RTF &amp; RWF) with the fastest treatment times actually have the highest reattendance rates in the dataset.</t>
   </si>
   <si>
     <t>#</t>
@@ -1380,12 +1380,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1395,11 +1410,26 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1407,11 +1437,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1949,22 +1988,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:C8"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="114.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="112.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2041,7 +2081,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:C12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.21875" bestFit="1" customWidth="1"/>
@@ -2049,14 +2089,15 @@
     <col min="3" max="3" width="99.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2190,89 +2231,89 @@
     <col min="28" max="28" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="4" t="s">
         <v>87</v>
       </c>
     </row>
@@ -14224,7 +14265,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:E13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -14234,20 +14275,21 @@
     <col min="5" max="5" width="63.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>379</v>
       </c>
     </row>
@@ -14472,31 +14514,32 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A2:D5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" style="5" customWidth="1"/>
     <col min="2" max="2" width="80.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="173" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="159.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>430</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
+      <c r="A3" s="5">
         <v>1</v>
       </c>
       <c r="B3" t="s">
@@ -14510,7 +14553,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
+      <c r="A4" s="5">
         <v>2</v>
       </c>
       <c r="B4" t="s">
@@ -14524,7 +14567,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5">
+      <c r="A5" s="5">
         <v>3</v>
       </c>
       <c r="B5" t="s">

</xml_diff>